<commit_message>
Update configuration files and enhance upload functionality
- Modified config.json to update SESSION_ID and Last run date.
- Updated emp_list.json to include new laboratory service personnel.
- Changed appendPool.html to add validation for tool code before saving.
- Added upload_delete_summary.txt to document the file upload/delete system architecture.
- Created tools_list.json as a new configuration file.
- Added filenames.csv to the reports directory with a list of lab identifiers.
- Updated Excel files for calibration records to reflect recent changes.
</commit_message>
<xml_diff>
--- a/py_test_ui/EXCEL FILE/recordCal_PM.xlsx
+++ b/py_test_ui/EXCEL FILE/recordCal_PM.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:Z22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,12 +568,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>216598</t>
+          <t>352896</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PYT3_06523</t>
+          <t>LAB-PY3-108</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -603,22 +603,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -686,11 +686,7 @@
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>PHYATHAI BEAUTY CENTER</t>
-        </is>
-      </c>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -700,12 +696,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>276701</t>
+          <t>353303</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PYT3_07564</t>
+          <t>LAB-PY3-112</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -735,22 +731,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -818,11 +814,2439 @@
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>X-RAY</t>
-        </is>
-      </c>
+      <c r="Z3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>353305</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>LAB-PY3-113</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>353306</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LAB-PY3-114</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>353307</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>LAB-PY3-115</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>353554</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>LAB-PY3-117</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>353555</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>LAB-PY3-118</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>353557</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>LAB-PY3-120</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>353573</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>LAB-PY3-126</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>354754</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>LAB-PY3-129</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>354755</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LAB-PY3-130</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>354756</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>LAB-PY3-131</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>354786</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LAB-PY3-138</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>400627</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>LAB-PY3-152</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>400633</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>LAB-PY3-154</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>400634</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>LAB-PY3-155</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>406508</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>LAB-PY3-159</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>428923</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>LAB-PY3-166</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>428924</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>LAB-PY3-167</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>428925</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>LAB-PY3-168</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>428926</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>LAB-PY3-169</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BME</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SOM KONKAEW</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>577199</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>DARANPHOP YIMYAM</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>PM doable</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Perform CAL</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>